<commit_message>
Corrida | SFE-ESC2 | 2026-06-17 11:32:43.251073
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ESC2_out.xlsx
+++ b/indicadores/SFE-ESC2_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="418">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Escrituras de ventas de la 2da circunscripción de Santa Fe (Sur)</t>
+    <t xml:space="preserve">Escrituras de ventas de la 2da circunscripción de Santa Fe</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sur de la provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">20/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1764,9 +1770,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1777,7 +1787,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1791,12 +1801,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.309078102888027</v>
+        <v>0.31167244210151</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1807,7 +1817,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1835,7 +1845,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1849,12 +1859,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.0895977683065296</v>
+        <v>0.0922937247258538</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1877,7 +1887,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1891,7 +1901,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1905,7 +1915,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1919,12 +1929,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00438338325468699</v>
+        <v>0.0056109700401958</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1935,7 +1945,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1949,12 +1959,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000102416675532499</v>
+        <v>0.000113240716308259</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2097,10 +2107,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2113,10 +2123,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2140,66 +2150,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>1657</v>
@@ -2252,7 +2262,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>1852</v>
@@ -2309,7 +2319,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>2242</v>
@@ -2366,7 +2376,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>2063</v>
@@ -2423,7 +2433,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>711</v>
@@ -2480,7 +2490,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>1824</v>
@@ -2537,7 +2547,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>2635</v>
@@ -2594,7 +2604,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>1959</v>
@@ -2651,7 +2661,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>1978</v>
@@ -2708,7 +2718,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>1579</v>
@@ -2765,7 +2775,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>2153</v>
@@ -2822,7 +2832,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>2561</v>
@@ -2879,7 +2889,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>1195</v>
@@ -2938,7 +2948,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>1364</v>
@@ -2997,7 +3007,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>1817</v>
@@ -3056,7 +3066,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>1896</v>
@@ -3115,7 +3125,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>1957</v>
@@ -3174,7 +3184,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>2033</v>
@@ -3233,7 +3243,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>1957</v>
@@ -3292,7 +3302,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>1968</v>
@@ -3351,7 +3361,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>2223</v>
@@ -3410,7 +3420,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>1899</v>
@@ -3469,7 +3479,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>1817</v>
@@ -3528,7 +3538,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>2502</v>
@@ -3587,7 +3597,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>1376</v>
@@ -3646,7 +3656,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>1407</v>
@@ -3705,7 +3715,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>1908</v>
@@ -3764,7 +3774,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>1850</v>
@@ -3823,7 +3833,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>1981</v>
@@ -3882,7 +3892,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>2104</v>
@@ -3941,7 +3951,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>1984</v>
@@ -4000,7 +4010,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>2300</v>
@@ -4059,7 +4069,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>2213</v>
@@ -4118,7 +4128,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>2264</v>
@@ -4177,7 +4187,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>1991</v>
@@ -4236,7 +4246,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>2177</v>
@@ -4295,7 +4305,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>1378</v>
@@ -4354,7 +4364,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>2266</v>
@@ -4413,7 +4423,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>2629</v>
@@ -4472,7 +4482,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>1697</v>
@@ -4531,7 +4541,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>1407</v>
@@ -4590,7 +4600,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>2367</v>
@@ -4649,7 +4659,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>2041</v>
@@ -4708,7 +4718,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>2478</v>
@@ -4767,7 +4777,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>2103</v>
@@ -4826,7 +4836,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>2126</v>
@@ -4885,7 +4895,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>1891</v>
@@ -4944,7 +4954,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>3212</v>
@@ -5003,7 +5013,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>1207</v>
@@ -5062,7 +5072,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>1605</v>
@@ -5121,7 +5131,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>1817</v>
@@ -5180,7 +5190,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>2012</v>
@@ -5239,7 +5249,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>2257</v>
@@ -5298,7 +5308,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>1854</v>
@@ -5357,7 +5367,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>2069</v>
@@ -5416,7 +5426,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>1856</v>
@@ -5475,7 +5485,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>1995</v>
@@ -5534,7 +5544,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>1908</v>
@@ -5593,7 +5603,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>1924</v>
@@ -5652,7 +5662,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>2079</v>
@@ -5711,7 +5721,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>795</v>
@@ -5770,7 +5780,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>1072</v>
@@ -5829,7 +5839,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>1471</v>
@@ -5888,7 +5898,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>1403</v>
@@ -5947,7 +5957,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>1405</v>
@@ -6006,7 +6016,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>1509</v>
@@ -6065,7 +6075,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>1480</v>
@@ -6124,7 +6134,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>1634</v>
@@ -6183,7 +6193,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>1750</v>
@@ -6242,7 +6252,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>1702</v>
@@ -6301,7 +6311,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>1631</v>
@@ -6360,7 +6370,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>2139</v>
@@ -6419,7 +6429,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>973</v>
@@ -6478,7 +6488,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>1110</v>
@@ -6537,7 +6547,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>1142</v>
@@ -6596,7 +6606,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>2046</v>
@@ -6655,7 +6665,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>1798</v>
@@ -6714,7 +6724,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>1673</v>
@@ -6773,7 +6783,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>2141</v>
@@ -6832,7 +6842,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>1611</v>
@@ -6891,7 +6901,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>1865</v>
@@ -6950,7 +6960,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>1696</v>
@@ -7009,7 +7019,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>2209</v>
@@ -7068,7 +7078,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>2351</v>
@@ -7127,7 +7137,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>1048</v>
@@ -7186,7 +7196,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>1245</v>
@@ -7245,7 +7255,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>1431</v>
@@ -7304,7 +7314,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>2133</v>
@@ -7363,7 +7373,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>2018</v>
@@ -7422,7 +7432,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>2104</v>
@@ -7481,7 +7491,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>3038</v>
@@ -7540,7 +7550,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>2248</v>
@@ -7599,7 +7609,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>2232</v>
@@ -7658,7 +7668,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>1952</v>
@@ -7717,7 +7727,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>2095</v>
@@ -7776,7 +7786,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>2592</v>
@@ -7835,7 +7845,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>1247</v>
@@ -7894,7 +7904,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>1157</v>
@@ -7953,7 +7963,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>1855</v>
@@ -8012,7 +8022,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>1501</v>
@@ -8071,7 +8081,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>1853</v>
@@ -8130,7 +8140,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>1792</v>
@@ -8189,7 +8199,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>1707</v>
@@ -8248,7 +8258,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>1940</v>
@@ -8307,7 +8317,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>1655</v>
@@ -8366,7 +8376,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>1668</v>
@@ -8425,7 +8435,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>1717</v>
@@ -8484,7 +8494,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>1779</v>
@@ -8543,7 +8553,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>939</v>
@@ -8602,7 +8612,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>1000</v>
@@ -8661,7 +8671,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>1635</v>
@@ -8720,7 +8730,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>1414</v>
@@ -8779,7 +8789,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>1939</v>
@@ -8838,7 +8848,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>1650</v>
@@ -8897,7 +8907,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>1715</v>
@@ -8956,7 +8966,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>1767</v>
@@ -9015,7 +9025,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>1748</v>
@@ -9074,7 +9084,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>1803</v>
@@ -9133,7 +9143,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>1784</v>
@@ -9192,7 +9202,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>1955</v>
@@ -9251,7 +9261,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>1567</v>
@@ -9310,7 +9320,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>1120</v>
@@ -9369,7 +9379,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>1369</v>
@@ -9428,7 +9438,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>1514</v>
@@ -9487,7 +9497,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>1363</v>
@@ -9546,7 +9556,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>1541</v>
@@ -9605,7 +9615,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>1833</v>
@@ -9664,7 +9674,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>1630</v>
@@ -9723,7 +9733,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>1532</v>
@@ -9782,7 +9792,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>1679</v>
@@ -9841,7 +9851,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>1545</v>
@@ -9900,7 +9910,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>1530</v>
@@ -9959,7 +9969,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>1322</v>
@@ -10018,7 +10028,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>1055</v>
@@ -10077,7 +10087,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>1030</v>
@@ -10136,7 +10146,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>1277</v>
@@ -10195,7 +10205,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>1457</v>
@@ -10254,7 +10264,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>1313</v>
@@ -10313,7 +10323,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>1151</v>
@@ -10372,7 +10382,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>1499</v>
@@ -10431,7 +10441,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>1400</v>
@@ -10490,7 +10500,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>1184</v>
@@ -10549,7 +10559,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>1593</v>
@@ -10608,7 +10618,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>1362</v>
@@ -10667,7 +10677,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>968</v>
@@ -10726,7 +10736,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>726</v>
@@ -10785,7 +10795,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>1075</v>
@@ -10844,7 +10854,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>1185</v>
@@ -10903,7 +10913,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>1136</v>
@@ -10962,7 +10972,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>1312</v>
@@ -11021,7 +11031,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>924</v>
@@ -11080,7 +11090,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>1241</v>
@@ -11139,7 +11149,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>1398</v>
@@ -11198,7 +11208,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>1442</v>
@@ -11257,7 +11267,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>1414</v>
@@ -11316,7 +11326,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>1515</v>
@@ -11375,7 +11385,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>1260</v>
@@ -11434,7 +11444,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>887</v>
@@ -11493,7 +11503,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>1278</v>
@@ -11552,7 +11562,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>987</v>
@@ -11611,7 +11621,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>1307</v>
@@ -11670,7 +11680,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>1700</v>
@@ -11729,7 +11739,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>1418</v>
@@ -11788,7 +11798,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>858</v>
@@ -11847,7 +11857,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>1736</v>
@@ -11906,7 +11916,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>1390</v>
@@ -11965,7 +11975,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>1855</v>
@@ -12024,7 +12034,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>1562</v>
@@ -12083,7 +12093,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>1306</v>
@@ -12142,7 +12152,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>1255</v>
@@ -12201,7 +12211,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>1489</v>
@@ -12260,7 +12270,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>1587</v>
@@ -12319,7 +12329,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>1666</v>
@@ -12378,7 +12388,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>1865</v>
@@ -12437,7 +12447,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>1383</v>
@@ -12496,7 +12506,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>1307</v>
@@ -12555,7 +12565,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>1099</v>
@@ -12614,7 +12624,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>1011</v>
@@ -12673,7 +12683,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>1536</v>
@@ -12732,7 +12742,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>1472</v>
@@ -12791,7 +12801,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>1166</v>
@@ -12850,7 +12860,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>1017</v>
@@ -12909,7 +12919,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>1041</v>
@@ -12968,7 +12978,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>1216</v>
@@ -13027,7 +13037,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>1179</v>
@@ -13086,7 +13096,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>1242</v>
@@ -13145,7 +13155,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>1037</v>
@@ -13204,7 +13214,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>1266</v>
@@ -13263,7 +13273,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>1137</v>
@@ -13322,7 +13332,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>923</v>
@@ -13381,7 +13391,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>678</v>
@@ -13440,7 +13450,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>1118</v>
@@ -13499,7 +13509,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>1162</v>
@@ -13558,7 +13568,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>799</v>
@@ -13617,7 +13627,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>844</v>
@@ -13676,7 +13686,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>201</v>
@@ -13735,7 +13745,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>102</v>
@@ -13794,7 +13804,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>568</v>
@@ -13853,7 +13863,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>701</v>
@@ -13912,7 +13922,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>1060</v>
@@ -13971,7 +13981,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>1184</v>
@@ -14030,7 +14040,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>709</v>
@@ -14089,7 +14099,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>1236</v>
@@ -14148,7 +14158,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>1250</v>
@@ -14207,7 +14217,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>1336</v>
@@ -14266,7 +14276,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>891</v>
@@ -14325,7 +14335,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>1471</v>
@@ -14384,7 +14394,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>1225</v>
@@ -14443,7 +14453,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>816</v>
@@ -14502,7 +14512,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>919</v>
@@ -14561,7 +14571,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>1365</v>
@@ -14620,7 +14630,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>1062</v>
@@ -14679,7 +14689,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>1183</v>
@@ -14738,7 +14748,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>1189</v>
@@ -14797,7 +14807,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>1195</v>
@@ -14856,7 +14866,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>1022</v>
@@ -14915,7 +14925,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>1075</v>
@@ -14974,7 +14984,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>789</v>
@@ -15033,7 +15043,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>1134</v>
@@ -15092,7 +15102,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>1333</v>
@@ -15151,7 +15161,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>1149</v>
@@ -15210,7 +15220,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>1125</v>
@@ -15269,7 +15279,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>1278</v>
@@ -15328,7 +15338,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>1167</v>
@@ -15387,7 +15397,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>1173</v>
@@ -15446,7 +15456,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>1450</v>
@@ -15505,7 +15515,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>1282</v>
@@ -15564,7 +15574,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>1322</v>
@@ -15623,7 +15633,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>1232</v>
@@ -15682,7 +15692,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>903</v>
@@ -15741,7 +15751,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>935</v>
@@ -15800,7 +15810,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>1349</v>
@@ -15859,7 +15869,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>1054</v>
@@ -15918,7 +15928,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>1242</v>
@@ -15977,7 +15987,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>1016</v>
@@ -16036,7 +16046,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>1263</v>
@@ -16095,7 +16105,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>1252</v>
@@ -16154,7 +16164,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>1525</v>
@@ -16213,7 +16223,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>887</v>
@@ -16272,7 +16282,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>1326</v>
@@ -16331,7 +16341,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>965</v>
@@ -16390,7 +16400,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>929</v>
@@ -16449,7 +16459,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>346</v>
@@ -16508,7 +16518,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>740</v>
@@ -16567,7 +16577,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>1276</v>
@@ -16626,7 +16636,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>1602</v>
@@ -16685,7 +16695,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>961</v>
@@ -16744,7 +16754,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>1614</v>
@@ -16803,7 +16813,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>1360</v>
@@ -16862,7 +16872,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>1820</v>
@@ -16921,7 +16931,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>1430</v>
@@ -16980,7 +16990,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>1486</v>
@@ -17039,7 +17049,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>1571</v>
@@ -17098,7 +17108,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>1387</v>
@@ -17157,7 +17167,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>1406</v>
@@ -17216,7 +17226,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>1725</v>
@@ -17275,7 +17285,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>1473</v>
@@ -17334,7 +17344,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>2789</v>
@@ -17393,7 +17403,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>1989</v>
@@ -17452,7 +17462,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>1782</v>
@@ -17511,7 +17521,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>2002</v>
@@ -17570,7 +17580,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>2054</v>
@@ -17629,7 +17639,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>1666</v>
@@ -17688,7 +17698,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>2172</v>
@@ -17747,7 +17757,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>1133</v>
@@ -17806,7 +17816,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>1266</v>
@@ -17865,7 +17875,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>1844</v>
@@ -17924,7 +17934,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2"/>
       <c r="C269" s="3" t="n">
@@ -17957,7 +17967,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2"/>
       <c r="C270" s="3" t="n">
@@ -17990,7 +18000,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2"/>
       <c r="C271" s="3" t="n">
@@ -18023,7 +18033,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2"/>
       <c r="C272" s="3" t="n">
@@ -18056,7 +18066,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2"/>
       <c r="C273" s="3" t="n">
@@ -18089,7 +18099,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2"/>
       <c r="C274" s="3" t="n">
@@ -18122,7 +18132,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2"/>
       <c r="C275" s="3" t="n">
@@ -18155,7 +18165,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2"/>
       <c r="C276" s="3" t="n">
@@ -18188,7 +18198,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2"/>
       <c r="C277" s="3" t="n">
@@ -18221,7 +18231,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2"/>
       <c r="C278" s="3" t="n">
@@ -18254,7 +18264,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2"/>
       <c r="C279" s="3" t="n">
@@ -18287,7 +18297,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2"/>
       <c r="C280" s="3" t="n">
@@ -18320,7 +18330,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2"/>
       <c r="C281" s="3"/>
@@ -18343,7 +18353,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2"/>
       <c r="C282" s="3"/>
@@ -18366,7 +18376,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2"/>
       <c r="C283" s="3"/>
@@ -18389,7 +18399,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2"/>
       <c r="C284" s="3"/>
@@ -18412,7 +18422,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2"/>
       <c r="C285" s="3"/>
@@ -18435,7 +18445,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2"/>
       <c r="C286" s="3"/>
@@ -18458,7 +18468,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2"/>
       <c r="C287" s="3"/>
@@ -18481,7 +18491,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2"/>
       <c r="C288" s="3"/>
@@ -18504,7 +18514,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2"/>
       <c r="C289" s="3"/>
@@ -18527,7 +18537,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2"/>
       <c r="C290" s="3"/>
@@ -18550,7 +18560,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2"/>
       <c r="C291" s="3"/>
@@ -18573,7 +18583,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2"/>
       <c r="C292" s="3"/>
@@ -18596,7 +18606,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2"/>
       <c r="C293" s="3"/>
@@ -18619,7 +18629,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2"/>
       <c r="C294" s="3"/>
@@ -18642,7 +18652,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2"/>
       <c r="C295" s="3"/>
@@ -18665,7 +18675,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2"/>
       <c r="C296" s="3"/>
@@ -18688,7 +18698,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2"/>
       <c r="C297" s="3"/>
@@ -18711,7 +18721,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2"/>
       <c r="C298" s="3"/>
@@ -18734,7 +18744,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2"/>
       <c r="C299" s="3"/>
@@ -18757,7 +18767,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2"/>
       <c r="C300" s="3"/>
@@ -18780,7 +18790,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2"/>
       <c r="C301" s="3"/>
@@ -18803,7 +18813,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2"/>
       <c r="C302" s="3"/>
@@ -18826,7 +18836,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2"/>
       <c r="C303" s="3"/>
@@ -18849,7 +18859,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2"/>
       <c r="C304" s="3"/>
@@ -18872,7 +18882,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2"/>
       <c r="C305" s="3"/>
@@ -18895,7 +18905,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2"/>
       <c r="C306" s="3"/>
@@ -18918,7 +18928,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2"/>
       <c r="C307" s="3"/>
@@ -18941,7 +18951,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2"/>
       <c r="C308" s="3"/>
@@ -18964,7 +18974,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2"/>
       <c r="C309" s="3"/>
@@ -18987,7 +18997,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2"/>
       <c r="C310" s="3"/>
@@ -19010,7 +19020,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2"/>
       <c r="C311" s="3"/>
@@ -19033,7 +19043,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2"/>
       <c r="C312" s="3"/>
@@ -19056,7 +19066,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2"/>
       <c r="C313" s="3"/>
@@ -19079,7 +19089,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2"/>
       <c r="C314" s="3"/>
@@ -19102,7 +19112,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2"/>
       <c r="C315" s="3"/>
@@ -19125,7 +19135,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2"/>
       <c r="C316" s="3"/>
@@ -19148,7 +19158,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2"/>
       <c r="C317" s="3"/>
@@ -19171,7 +19181,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2"/>
       <c r="C318" s="3"/>
@@ -19194,7 +19204,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2"/>
       <c r="C319" s="3"/>
@@ -19217,7 +19227,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2"/>
       <c r="C320" s="3"/>
@@ -19240,7 +19250,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2"/>
       <c r="C321" s="3"/>
@@ -19263,7 +19273,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2"/>
       <c r="C322" s="3"/>
@@ -19286,7 +19296,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2"/>
       <c r="C323" s="3"/>
@@ -19309,7 +19319,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2"/>
       <c r="C324" s="3"/>
@@ -19332,7 +19342,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2"/>
       <c r="C325" s="3"/>
@@ -19366,97 +19376,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -19480,7 +19490,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -19490,160 +19500,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0997814953201027</v>
+        <v>-0.0995414174653064</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0290806668158503</v>
+        <v>-0.0294660128066697</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0315368777575713</v>
+        <v>0.0318834253256469</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.075151831905511</v>
+        <v>0.0729198150715978</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.0204951377839295</v>
+        <v>0.0177307721453943</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.0490967439667967</v>
+        <v>0.0480490547287371</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.215170677917852</v>
+        <v>0.213512062525735</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.297115932800192</v>
+        <v>0.295404252710187</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.289374181597557</v>
+        <v>0.291287220687535</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.2993288631364</v>
+        <v>0.303798822785497</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.309078102888027</v>
+        <v>0.31167244210151</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.250346077482383</v>
+        <v>0.250478819311447</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.147769248149946</v>
+        <v>0.14676805988633</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.09213272037801</v>
+        <v>0.0918886823892788</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0696036687703921</v>
+        <v>0.0712362499041025</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>-0.0127883762130812</v>
+        <v>-0.00962224664171196</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.094625866678356</v>
+        <v>-0.0915590583645573</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.142912379885737</v>
+        <v>-0.141577131258509</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.20540868569958</v>
+        <v>-0.20510197308878</v>
       </c>
     </row>
     <row r="24">

</xml_diff>